<commit_message>
Divided MgmtIndex_ProvaBrasil_StdtYear.dta into 15 parts, updated README and replication_files
</commit_message>
<xml_diff>
--- a/replication_files.xlsx
+++ b/replication_files.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\~Variados\Files transfer folder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C604A67-67DB-4757-BE17-38EFAA873670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EBD9060-0539-477C-BE5D-7AC7338CD1BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Replication Files" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1226" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="375">
   <si>
     <t>root</t>
   </si>
@@ -1144,6 +1144,9 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>cleaning/1_pb_cleaning.do (divided into 15 parts due to size limitations)</t>
   </si>
 </sst>
 </file>
@@ -1499,9 +1502,11 @@
   <dimension ref="A1:H156"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="57.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="57.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.88671875" customWidth="1"/>
-    <col min="6" max="6" width="38.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="60.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="74.5546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -1539,6 +1544,9 @@
       <c r="D2" t="s">
         <v>9</v>
       </c>
+      <c r="E2" t="s">
+        <v>173</v>
+      </c>
       <c r="H2" t="s">
         <v>9</v>
       </c>
@@ -1547,6 +1555,9 @@
       <c r="D3" t="s">
         <v>10</v>
       </c>
+      <c r="E3" t="s">
+        <v>173</v>
+      </c>
       <c r="H3" t="s">
         <v>10</v>
       </c>
@@ -3103,7 +3114,7 @@
         <v>214</v>
       </c>
       <c r="F98" t="s">
-        <v>174</v>
+        <v>374</v>
       </c>
       <c r="H98" t="s">
         <v>216</v>
@@ -4162,10 +4173,10 @@
   <dimension ref="A1:D76"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="48.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="74.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -5242,9 +5253,9 @@
   <dimension ref="A1:D36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>